<commit_message>
feat: remove Anthropic from Act 1, use fixed scripts + direct testimonials
Act 1 now uses fixed text files for the director speech and client
testimonials instead of Anthropic-generated content. Anthropic API is
retained only for the council phase (minute 45).

- Add fixed director speech (guiones/director.txt) and Adriana Rueda
  role-explanation script (guiones/adriana.txt)
- Rewrite anthropic.ts: remove generarDiscursoDirector/generarParlamentosClientes,
  add generarParlamentosDirectos that passes comment text through directly
- Add Adriana as new character in escena.ts with dedicated voice config
- Update sala.ts to serve adriana piece in escena:solicitar/escena:audio
- Add startup validation of fixed text against prohibited terms
- Copy corrected Excel comments file
- All 21 data verifications pass, TypeScript compiles clean

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0118D8TUxwMpU8NFigARUZyD
</commit_message>
<xml_diff>
--- a/datos/R2_ETF_Bank_Comentarios_Clientes.xlsx
+++ b/datos/R2_ETF_Bank_Comentarios_Clientes.xlsx
@@ -582,7 +582,7 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Entregue todo lo que me pidieron y aun asi hubo 3 rondas de correcciones. Es desgastante.</t>
+          <t>Entregué todo lo que me pidieron y aun así hubo 3 rondas de correcciones. Es desgastante.</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -629,7 +629,7 @@
       <c r="I6" s="4" t="inlineStr"/>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Despues de 3 intentos ya perdi la cuenta de cuantas copias de mi identificacion he entregado.</t>
+          <t>Después de 3 intentos ya perdí la cuenta de cuántas copias de mi identificación he entregado.</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Pedi la tarjeta el 5 de abril. Entre correcciones y papeles faltantes llevo 53 dias esperando.</t>
+          <t>Pedí la tarjeta el 5 de abril. Entre correcciones y papeles faltantes llevo 53 días esperando.</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -727,7 +727,7 @@
       <c r="I8" s="4" t="inlineStr"/>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Me pidieron documentos incompletos en dos ocasiones distintas, con semanas de diferencia. Si faltaba algo, dimelo desde el principio.</t>
+          <t>Me pidieron documentos incompletos en dos ocasiones distintas, con semanas de diferencia. Si faltaba algo, dímelo desde el principio.</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -1029,7 +1029,7 @@
       <c r="I14" s="4" t="inlineStr"/>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Despues de 3 intentos ya perdi la cuenta de cuantas copias de mi identificacion he entregado.</t>
+          <t>Después de 3 intentos ya perdí la cuenta de cuántas copias de mi identificación he entregado.</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
@@ -1123,7 +1123,7 @@
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Me hicieron volver 3 veces por documentos. Trabajo y cada visita me cuesta medio dia.</t>
+          <t>Me hicieron volver 3 veces por documentos. Trabajo y cada visita me cuesta medio día.</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Me pidieron documentos incompletos en dos ocasiones distintas, con semanas de diferencia. Si faltaba algo, dimelo desde el principio.</t>
+          <t>Me pidieron documentos incompletos en dos ocasiones distintas, con semanas de diferencia. Si faltaba algo, dímelo desde el principio.</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       <c r="I20" s="4" t="inlineStr"/>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Me pidieron documentos incompletos en dos ocasiones distintas, con semanas de diferencia. Si faltaba algo, dimelo desde el principio.</t>
+          <t>Me pidieron documentos incompletos en dos ocasiones distintas, con semanas de diferencia. Si faltaba algo, dímelo desde el principio.</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Pedi la tarjeta el 19 de marzo. Entre correcciones y papeles faltantes llevo 37 dias esperando.</t>
+          <t>Pedí la tarjeta el 19 de marzo. Entre correcciones y papeles faltantes llevo 37 días esperando.</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Llevo 18 dias en este tramite y 3 entregas de documentos. No entiendo por que no revisan todo junto la primera vez.</t>
+          <t>Llevo 18 días en este trámite y 3 entregas de documentos. No entiendo por qué no revisan todo junto la primera vez.</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Entregue todo lo que me pidieron y aun asi hubo 4 rondas de correcciones. Es desgastante.</t>
+          <t>Entregué todo lo que me pidieron y aun así hubo 4 rondas de correcciones. Es desgastante.</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
@@ -1570,7 +1570,7 @@
       <c r="I25" s="4" t="inlineStr"/>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>Llevo 30 dias en este tramite y 3 entregas de documentos. No entiendo por que no revisan todo junto la primera vez.</t>
+          <t>Llevo 30 días en este trámite y 3 entregas de documentos. No entiendo por qué no revisan todo junto la primera vez.</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
@@ -1617,7 +1617,7 @@
       <c r="I26" s="4" t="inlineStr"/>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>Me hicieron volver 3 veces por documentos. Trabajo y cada visita me cuesta medio dia.</t>
+          <t>Me hicieron volver 3 veces por documentos. Trabajo y cada visita me cuesta medio día.</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>Me pidieron documentos incompletos en dos ocasiones distintas, con semanas de diferencia. Si faltaba algo, dimelo desde el principio.</t>
+          <t>Me pidieron documentos incompletos en dos ocasiones distintas, con semanas de diferencia. Si faltaba algo, dímelo desde el principio.</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>Llevo 46 dias en este tramite y 3 entregas de documentos. No entiendo por que no revisan todo junto la primera vez.</t>
+          <t>Llevo 46 días en este trámite y 3 entregas de documentos. No entiendo por qué no revisan todo junto la primera vez.</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>Me pidieron documentos incompletos en dos ocasiones distintas, con semanas de diferencia. Si faltaba algo, dimelo desde el principio.</t>
+          <t>Me pidieron documentos incompletos en dos ocasiones distintas, con semanas de diferencia. Si faltaba algo, dímelo desde el principio.</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr">
@@ -1817,7 +1817,7 @@
       <c r="I30" s="4" t="inlineStr"/>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>Llevo 34 dias en este tramite y 3 entregas de documentos. No entiendo por que no revisan todo junto la primera vez.</t>
+          <t>Llevo 34 días en este trámite y 3 entregas de documentos. No entiendo por qué no revisan todo junto la primera vez.</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>Me hicieron volver 3 veces por documentos. Trabajo y cada visita me cuesta medio dia.</t>
+          <t>Me hicieron volver 3 veces por documentos. Trabajo y cada visita me cuesta medio día.</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>Despues de 4 intentos ya perdi la cuenta de cuantas copias de mi identificacion he entregado.</t>
+          <t>Después de 4 intentos ya perdí la cuenta de cuántas copias de mi identificación he entregado.</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>Pedi la tarjeta el 12 de agosto. Entre correcciones y papeles faltantes llevo 69 dias esperando.</t>
+          <t>Pedí la tarjeta el 12 de agosto. Entre correcciones y papeles faltantes llevo 69 días esperando.</t>
         </is>
       </c>
       <c r="K37" s="4" t="inlineStr">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>Llevo 54 dias en este tramite y 4 entregas de documentos. No entiendo por que no revisan todo junto la primera vez.</t>
+          <t>Llevo 54 días en este trámite y 4 entregas de documentos. No entiendo por qué no revisan todo junto la primera vez.</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>Llevo 52 dias en este tramite y 3 entregas de documentos. No entiendo por que no revisan todo junto la primera vez.</t>
+          <t>Llevo 52 días en este trámite y 3 entregas de documentos. No entiendo por qué no revisan todo junto la primera vez.</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
@@ -2413,7 +2413,7 @@
       <c r="I42" s="4" t="inlineStr"/>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>Entregue todo lo que me pidieron y aun asi hubo 3 rondas de correcciones. Es desgastante.</t>
+          <t>Entregué todo lo que me pidieron y aun así hubo 3 rondas de correcciones. Es desgastante.</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>Despues de 3 intentos ya perdi la cuenta de cuantas copias de mi identificacion he entregado.</t>
+          <t>Después de 3 intentos ya perdí la cuenta de cuántas copias de mi identificación he entregado.</t>
         </is>
       </c>
       <c r="K45" s="4" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
-          <t>Revisaron mi solicitud y encontraron errores de captura del propio banco. Y me toco esperar de nuevo.</t>
+          <t>Revisaron mi solicitud y encontraron errores de captura del propio banco. Y me tocó esperar de nuevo.</t>
         </is>
       </c>
       <c r="K48" s="4" t="inlineStr">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>Revisaron mi solicitud y encontraron errores de captura del propio banco. Y me toco esperar de nuevo.</t>
+          <t>Revisaron mi solicitud y encontraron errores de captura del propio banco. Y me tocó esperar de nuevo.</t>
         </is>
       </c>
       <c r="K49" s="4" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>Mi domicilio quedo mal registrado y eso atraso todo 74 dias. Fue un error de ellos, no mio.</t>
+          <t>Mi domicilio quedó mal registrado y eso atrasó todo 74 días. Fue un error de ellos, no mío.</t>
         </is>
       </c>
       <c r="K51" s="4" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
-          <t>Revisaron mi solicitud y encontraron errores de captura del propio banco. Y me toco esperar de nuevo.</t>
+          <t>Revisaron mi solicitud y encontraron errores de captura del propio banco. Y me tocó esperar de nuevo.</t>
         </is>
       </c>
       <c r="K53" s="4" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="J54" s="4" t="inlineStr">
         <is>
-          <t>Revisaron mi solicitud y encontraron errores de captura del propio banco. Y me toco esperar de nuevo.</t>
+          <t>Revisaron mi solicitud y encontraron errores de captura del propio banco. Y me tocó esperar de nuevo.</t>
         </is>
       </c>
       <c r="K54" s="4" t="inlineStr">
@@ -3072,7 +3072,7 @@
       </c>
       <c r="J55" s="4" t="inlineStr">
         <is>
-          <t>Revisaron mi solicitud y encontraron errores de captura del propio banco. Y me toco esperar de nuevo.</t>
+          <t>Revisaron mi solicitud y encontraron errores de captura del propio banco. Y me tocó esperar de nuevo.</t>
         </is>
       </c>
       <c r="K55" s="4" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
-          <t>Capturaron mal mi informacion y por eso se rechazo el primer intento. Nadie me aviso, yo tuve que preguntar.</t>
+          <t>Capturaron mal mi información y por eso se rechazó el primer intento. Nadie me avisó, yo tuve que preguntar.</t>
         </is>
       </c>
       <c r="K56" s="4" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="J60" s="4" t="inlineStr">
         <is>
-          <t>Mi solicitud fue autorizada y ahi se quedo. No hay tarjeta, no hay explicacion, no hay a quien preguntar.</t>
+          <t>Mi solicitud fue autorizada y ahi se quedó. No hay tarjeta, no hay explicación, no hay a quien preguntar.</t>
         </is>
       </c>
       <c r="K60" s="4" t="inlineStr">
@@ -3378,7 +3378,7 @@
       </c>
       <c r="J61" s="4" t="inlineStr">
         <is>
-          <t>Mi solicitud fue autorizada y ahi se quedo. No hay tarjeta, no hay explicacion, no hay a quien preguntar.</t>
+          <t>Mi solicitud fue autorizada y ahi se quedó. No hay tarjeta, no hay explicación, no hay a quien preguntar.</t>
         </is>
       </c>
       <c r="K61" s="4" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="J62" s="4" t="inlineStr">
         <is>
-          <t>Me autorizaron y nadie me ha vuelto a llamar. Cuando marco me dicen que esta en proceso, sin mas detalle.</t>
+          <t>Me autorizaron y nadie me ha vuelto a llamar. Cuando marco me dicen que está en proceso, sin más detalle.</t>
         </is>
       </c>
       <c r="K62" s="4" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="J63" s="4" t="inlineStr">
         <is>
-          <t>Aprobaron mi credito y luego silencio total. Ya no se si cancelar o seguir esperando.</t>
+          <t>Aprobaron mi crédito y luego silencio total. Ya no se si cancelar o seguir esperando.</t>
         </is>
       </c>
       <c r="K63" s="4" t="inlineStr">
@@ -3574,7 +3574,7 @@
       <c r="I65" s="4" t="inlineStr"/>
       <c r="J65" s="4" t="inlineStr">
         <is>
-          <t>Mi solicitud fue autorizada y ahi se quedo. No hay tarjeta, no hay explicacion, no hay a quien preguntar.</t>
+          <t>Mi solicitud fue autorizada y ahi se quedó. No hay tarjeta, no hay explicación, no hay a quien preguntar.</t>
         </is>
       </c>
       <c r="K65" s="4" t="inlineStr">
@@ -3621,7 +3621,7 @@
       <c r="I66" s="4" t="inlineStr"/>
       <c r="J66" s="4" t="inlineStr">
         <is>
-          <t>Aprobaron mi credito y luego silencio total. Ya no se si cancelar o seguir esperando.</t>
+          <t>Aprobaron mi crédito y luego silencio total. Ya no se si cancelar o seguir esperando.</t>
         </is>
       </c>
       <c r="K66" s="4" t="inlineStr">
@@ -3672,7 +3672,7 @@
       </c>
       <c r="J67" s="4" t="inlineStr">
         <is>
-          <t>Aprobaron mi credito y luego silencio total. Ya no se si cancelar o seguir esperando.</t>
+          <t>Aprobaron mi crédito y luego silencio total. Ya no se si cancelar o seguir esperando.</t>
         </is>
       </c>
       <c r="K67" s="4" t="inlineStr">
@@ -3723,7 +3723,7 @@
       </c>
       <c r="J68" s="4" t="inlineStr">
         <is>
-          <t>Me confirmaron la aprobacion por telefono. De eso ya pasaron 46 dias y sigo sin tarjeta.</t>
+          <t>Me confirmaron la aprobación por teléfono. De eso ya pasaron 46 días y sigo sin tarjeta.</t>
         </is>
       </c>
       <c r="K68" s="4" t="inlineStr">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="J70" s="4" t="inlineStr">
         <is>
-          <t>Aprobaron mi credito y luego silencio total. Ya no se si cancelar o seguir esperando.</t>
+          <t>Aprobaron mi crédito y luego silencio total. Ya no se si cancelar o seguir esperando.</t>
         </is>
       </c>
       <c r="K70" s="4" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="J73" s="4" t="inlineStr">
         <is>
-          <t>Mas de dos meses de tramite. Si me hubieran dicho desde el inicio, no lo empiezo.</t>
+          <t>Mas de dos meses de trámite. Si me hubieran dicho desde el inicio, no lo empiezo.</t>
         </is>
       </c>
       <c r="K73" s="4" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="J74" s="4" t="inlineStr">
         <is>
-          <t>82 dias para una tarjeta. En ese tiempo ya cambie de necesidad, ya no me sirve.</t>
+          <t>82 días para una tarjeta. En ese tiempo ya cambié de necesidad, ya no me sirve.</t>
         </is>
       </c>
       <c r="K74" s="4" t="inlineStr">
@@ -4076,7 +4076,7 @@
       </c>
       <c r="J75" s="4" t="inlineStr">
         <is>
-          <t>El proceso se siente eterno. Nadie me da una fecha, solo me dicen que esta en revision.</t>
+          <t>El proceso se siente eterno. Nadie me da una fecha, solo me dicen que está en revisión.</t>
         </is>
       </c>
       <c r="K75" s="4" t="inlineStr">
@@ -4123,7 +4123,7 @@
       <c r="I76" s="4" t="inlineStr"/>
       <c r="J76" s="4" t="inlineStr">
         <is>
-          <t>70 dias para una tarjeta. En ese tiempo ya cambie de necesidad, ya no me sirve.</t>
+          <t>70 días para una tarjeta. En ese tiempo ya cambié de necesidad, ya no me sirve.</t>
         </is>
       </c>
       <c r="K76" s="4" t="inlineStr">
@@ -4170,7 +4170,7 @@
       <c r="I77" s="4" t="inlineStr"/>
       <c r="J77" s="4" t="inlineStr">
         <is>
-          <t>Mas de dos meses de tramite. Si me hubieran dicho desde el inicio, no lo empiezo.</t>
+          <t>Mas de dos meses de trámite. Si me hubieran dicho desde el inicio, no lo empiezo.</t>
         </is>
       </c>
       <c r="K77" s="4" t="inlineStr">
@@ -4221,7 +4221,7 @@
       </c>
       <c r="J78" s="4" t="inlineStr">
         <is>
-          <t>Entregue mi solicitud el 24 de octubre y todavia no se resuelve. Son 54 dias por una tarjeta de credito.</t>
+          <t>Entregué mi solicitud el 24 de octubre y todavia no se resuelve. Son 54 días por una tarjeta de crédito.</t>
         </is>
       </c>
       <c r="K78" s="4" t="inlineStr">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="J79" s="4" t="inlineStr">
         <is>
-          <t>En otro banco me resolvieron en una semana. Aqui llevo 57 dias.</t>
+          <t>En otro banco me resolvieron en una semana. Aqui llevo 57 días.</t>
         </is>
       </c>
       <c r="K79" s="4" t="inlineStr">
@@ -4323,7 +4323,7 @@
       </c>
       <c r="J80" s="4" t="inlineStr">
         <is>
-          <t>En otro banco me resolvieron en una semana. Aqui llevo 71 dias.</t>
+          <t>En otro banco me resolvieron en una semana. Aqui llevo 71 días.</t>
         </is>
       </c>
       <c r="K80" s="4" t="inlineStr">
@@ -4370,7 +4370,7 @@
       <c r="I81" s="4" t="inlineStr"/>
       <c r="J81" s="4" t="inlineStr">
         <is>
-          <t>Entregue mi solicitud el 9 de septiembre y todavia no se resuelve. Son 70 dias por una tarjeta de credito.</t>
+          <t>Entregué mi solicitud el 9 de septiembre y todavia no se resuelve. Son 70 días por una tarjeta de crédito.</t>
         </is>
       </c>
       <c r="K81" s="4" t="inlineStr">
@@ -4417,7 +4417,7 @@
       <c r="I82" s="4" t="inlineStr"/>
       <c r="J82" s="4" t="inlineStr">
         <is>
-          <t>70 dias para una tarjeta. En ese tiempo ya cambie de necesidad, ya no me sirve.</t>
+          <t>70 días para una tarjeta. En ese tiempo ya cambié de necesidad, ya no me sirve.</t>
         </is>
       </c>
       <c r="K82" s="4" t="inlineStr">
@@ -4468,7 +4468,7 @@
       </c>
       <c r="J83" s="4" t="inlineStr">
         <is>
-          <t>Rechazado despues de 3 intentos de entregar documentos. Nadie me explico el criterio.</t>
+          <t>Rechazado después de 3 intentos de entregar documentos. Nadie me explico el criterio.</t>
         </is>
       </c>
       <c r="K83" s="4" t="inlineStr">
@@ -4562,7 +4562,7 @@
       <c r="I85" s="4" t="inlineStr"/>
       <c r="J85" s="4" t="inlineStr">
         <is>
-          <t>Me hicieron correr por documentos durante 14 dias para al final decirme que no. Es una falta de respeto al tiempo del cliente.</t>
+          <t>Me hicieron correr por documentos durante 14 días para al final decirme que no. Es una falta de respeto al tiempo del cliente.</t>
         </is>
       </c>
       <c r="K85" s="4" t="inlineStr">
@@ -4609,7 +4609,7 @@
       <c r="I86" s="4" t="inlineStr"/>
       <c r="J86" s="4" t="inlineStr">
         <is>
-          <t>Rechazado despues de 2 intentos de entregar documentos. Nadie me explico el criterio.</t>
+          <t>Rechazado después de 2 intentos de entregar documentos. Nadie me explico el criterio.</t>
         </is>
       </c>
       <c r="K86" s="4" t="inlineStr">
@@ -4656,7 +4656,7 @@
       <c r="I87" s="4" t="inlineStr"/>
       <c r="J87" s="4" t="inlineStr">
         <is>
-          <t>Tengo 6 anos con el banco, buen historial, y me rechazaron por un puntaje que nadie me quiso explicar.</t>
+          <t>Tengo 6 años con el banco, buen historial, y me rechazaron por un puntaje que nadie me quiso explicar.</t>
         </is>
       </c>
       <c r="K87" s="4" t="inlineStr">
@@ -4754,7 +4754,7 @@
       </c>
       <c r="J89" s="4" t="inlineStr">
         <is>
-          <t>Rechazado despues de 4 intentos de entregar documentos. Nadie me explico el criterio.</t>
+          <t>Rechazado después de 4 intentos de entregar documentos. Nadie me explico el criterio.</t>
         </is>
       </c>
       <c r="K89" s="4" t="inlineStr">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="J90" s="4" t="inlineStr">
         <is>
-          <t>La linea que me dieron no corresponde a mi historial. Pedi explicacion y no me la dieron.</t>
+          <t>La linea que me dieron no corresponde a mi historial. Pedí explicación y no me la dieron.</t>
         </is>
       </c>
       <c r="K90" s="4" t="inlineStr">
@@ -4852,7 +4852,7 @@
       <c r="I91" s="4" t="inlineStr"/>
       <c r="J91" s="4" t="inlineStr">
         <is>
-          <t>1 rondas de documentos para que al final me autorizaran 28,000 pesos. No valio la pena el tramite.</t>
+          <t>1 rondas de documentos para que al final me autorizaran 28,000 pesos. No valió la pena el trámite.</t>
         </is>
       </c>
       <c r="K91" s="4" t="inlineStr">
@@ -4903,7 +4903,7 @@
       </c>
       <c r="J92" s="4" t="inlineStr">
         <is>
-          <t>Me aprobaron 31,400 pesos. Es la linea mas baja que me han ofrecido y ni me dijeron como la calcularon.</t>
+          <t>Me aprobaron 31,400 pesos. Es la linea más baja que me han ofrecido y ni me dijeron como la calcularon.</t>
         </is>
       </c>
       <c r="K92" s="4" t="inlineStr">
@@ -4950,7 +4950,7 @@
       <c r="I93" s="4" t="inlineStr"/>
       <c r="J93" s="4" t="inlineStr">
         <is>
-          <t>2 rondas de documentos para que al final me autorizaran 31,700 pesos. No valio la pena el tramite.</t>
+          <t>2 rondas de documentos para que al final me autorizaran 31,700 pesos. No valió la pena el trámite.</t>
         </is>
       </c>
       <c r="K93" s="4" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="J94" s="4" t="inlineStr">
         <is>
-          <t>La linea que me dieron no corresponde a mi historial. Pedi explicacion y no me la dieron.</t>
+          <t>La linea que me dieron no corresponde a mi historial. Pedí explicación y no me la dieron.</t>
         </is>
       </c>
       <c r="K94" s="4" t="inlineStr">

</xml_diff>